<commit_message>
refactored mail to fix mailno issue
</commit_message>
<xml_diff>
--- a/d_Mail/Import/HBT - Mail_Template.xlsx
+++ b/d_Mail/Import/HBT - Mail_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicole.millinship\PycharmProjects\AconexPython\d_Mail\Import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5EA53EF-0890-4C15-8D57-74FD76A6D482}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719D0FEC-BC9E-4C0E-A50D-FD7F50EA78B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="946" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -20,13 +20,17 @@
     <sheet name="10" sheetId="5" r:id="rId5"/>
     <sheet name="1879048689" sheetId="6" r:id="rId6"/>
     <sheet name="2198" sheetId="7" r:id="rId7"/>
+    <sheet name="23" sheetId="8" r:id="rId8"/>
+    <sheet name="1879048552" sheetId="9" r:id="rId9"/>
+    <sheet name="400" sheetId="10" r:id="rId10"/>
+    <sheet name="1879048558" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="39">
   <si>
     <t>(ECC) Early Warning Notice</t>
   </si>
@@ -34,13 +38,22 @@
     <t>1879048577</t>
   </si>
   <si>
+    <t>RowID*</t>
+  </si>
+  <si>
     <t>Mail Number (Leave blank for auto-number)</t>
   </si>
   <si>
+    <t>Email EntryID (Leave blank if no email)</t>
+  </si>
+  <si>
     <t>Reply to Mail Number (Leave blank for new thread)</t>
   </si>
   <si>
-    <t>To Names (Separate by semi-colon)</t>
+    <t>Reply to RowID (Use to reply to another imported mail)</t>
+  </si>
+  <si>
+    <t>To Names (Separate by semi-colon)*</t>
   </si>
   <si>
     <t>From Name (Leave blank for NM)</t>
@@ -49,7 +62,7 @@
     <t>CC Names (Separate by semi-colon)</t>
   </si>
   <si>
-    <t>Subject</t>
+    <t>Subject*</t>
   </si>
   <si>
     <t>Response Required Date</t>
@@ -112,25 +125,28 @@
     <t>2198</t>
   </si>
   <si>
-    <t>Dolph Lundgren</t>
-  </si>
-  <si>
-    <t>Nicole Millinship</t>
-  </si>
-  <si>
-    <t>Auto-Generated COR</t>
-  </si>
-  <si>
-    <t>Hi Dolph, can you read this?</t>
-  </si>
-  <si>
-    <t>To Names (Separate by semi-colon)*</t>
-  </si>
-  <si>
-    <t>Subject*</t>
-  </si>
-  <si>
-    <t>Anthony Apple; Bob Banana</t>
+    <t>Transmittal</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Extension of Time</t>
+  </si>
+  <si>
+    <t>1879048552</t>
+  </si>
+  <si>
+    <t>Workflow Transmittal</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>RFI Response</t>
+  </si>
+  <si>
+    <t>1879048558</t>
   </si>
 </sst>
 </file>
@@ -163,7 +179,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -171,34 +187,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,78 +508,75 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N2"/>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="14" width="30" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="L2" s="2" t="s">
         <v>13</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>15</v>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J3:J1000" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0900-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -587,65 +584,75 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J2"/>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J3:J1000" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -653,88 +660,88 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J3"/>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="17" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="G2" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G3" s="3">
-        <v>46101</v>
-      </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="b">
-        <v>1</v>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J3:J1000" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -742,72 +749,75 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:L2"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="12" width="30" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>23</v>
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J3:J1000" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -815,75 +825,75 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="13" width="30" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J3:J1000" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -891,69 +901,82 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:K2"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="80" customWidth="1"/>
-    <col min="9" max="9" width="30" customWidth="1"/>
-    <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="30" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="15" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>23</v>
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="J3:J1000" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -961,6 +984,324 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="16" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0500-000000000000}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="14" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0600-000000000000}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0700-000000000000}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="5" width="25" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="25" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="11" width="80" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000" xr:uid="{00000000-0002-0000-0800-000000000000}">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{428e5717-1df4-456d-8576-f827ff2d20e1}" enabled="1" method="Privileged" siteId="{69033406-071b-4a95-919c-befbd00ae24c}" contentBits="0" removed="0"/>

</xml_diff>